<commit_message>
doc(JitViewer): update tips for excel format file (#8097)
* doc: 更新 xlsx 文件移除图片

* doc: 增加已知问题
</commit_message>
<xml_diff>
--- a/src/BootstrapBlazor.Server/wwwroot/samples/sample.xlsx
+++ b/src/BootstrapBlazor.Server/wwwroot/samples/sample.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" checkCompatibility="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{694FDC00-D895-C449-B46D-4A0A3B3AE76D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="29400" windowHeight="17140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Invoice" sheetId="24" r:id="rId1"/>
@@ -179,9 +180,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.000%"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.000%"/>
   </numFmts>
   <fonts count="46" x14ac:knownFonts="1">
     <font>
@@ -1045,7 +1046,7 @@
     <xf numFmtId="43" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1055,7 +1056,7 @@
     <xf numFmtId="0" fontId="37" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="44" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1078,7 +1079,7 @@
     <xf numFmtId="0" fontId="44" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="44" fontId="44" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="44" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="34" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1231,63 +1232,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>1640417</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>492919</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="Vertex42 logo">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7315200" y="123825"/>
-          <a:ext cx="1640417" cy="369094"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1343,7 +1288,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/theme/theme11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Simple service invoice">
@@ -1544,26 +1489,26 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="B1:I44"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="3.796875" style="7" customWidth="1"/>
-    <col min="2" max="2" width="40.796875" style="7" customWidth="1"/>
-    <col min="3" max="3" width="10.796875" style="7" customWidth="1"/>
-    <col min="4" max="4" width="5.796875" style="7" customWidth="1"/>
-    <col min="5" max="6" width="18.796875" style="7" customWidth="1"/>
-    <col min="7" max="7" width="3.796875" style="7" customWidth="1"/>
+    <col min="1" max="1" width="3.83203125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" style="7" customWidth="1"/>
+    <col min="4" max="4" width="5.83203125" style="7" customWidth="1"/>
+    <col min="5" max="6" width="18.83203125" style="7" customWidth="1"/>
+    <col min="7" max="7" width="3.83203125" style="7" customWidth="1"/>
     <col min="8" max="8" width="29" style="7" customWidth="1"/>
     <col min="9" max="16384" width="9" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.9">
+    <row r="1" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:9" ht="46.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="B2" s="52" t="s">
         <v>0</v>
       </c>
@@ -1573,7 +1518,7 @@
       </c>
       <c r="F2" s="60"/>
     </row>
-    <row r="3" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="14" t="s">
         <v>2</v>
       </c>
@@ -1586,7 +1531,7 @@
       </c>
       <c r="I3" s="17"/>
     </row>
-    <row r="4" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="14" t="s">
         <v>4</v>
       </c>
@@ -1599,7 +1544,7 @@
       </c>
       <c r="I4" s="19"/>
     </row>
-    <row r="5" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="14" t="s">
         <v>6</v>
       </c>
@@ -1607,13 +1552,13 @@
       <c r="D5" s="21"/>
       <c r="H5" s="22"/>
     </row>
-    <row r="6" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="23"/>
       <c r="C6" s="18"/>
       <c r="D6" s="24"/>
       <c r="H6" s="22"/>
     </row>
-    <row r="7" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="62" t="s">
         <v>9</v>
       </c>
@@ -1629,7 +1574,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="25" t="s">
         <v>13</v>
       </c>
@@ -1640,11 +1585,11 @@
       </c>
       <c r="F8" s="27">
         <f ca="1">TODAY()</f>
-        <v>45679</v>
+        <v>46182</v>
       </c>
       <c r="H8" s="22"/>
     </row>
-    <row r="9" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="25" t="s">
         <v>15</v>
       </c>
@@ -1654,7 +1599,7 @@
       <c r="F9" s="27"/>
       <c r="H9" s="16"/>
     </row>
-    <row r="10" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="25" t="s">
         <v>16</v>
       </c>
@@ -1668,7 +1613,7 @@
       </c>
       <c r="H10" s="16"/>
     </row>
-    <row r="11" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="25" t="s">
         <v>17</v>
       </c>
@@ -1684,7 +1629,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="25" t="s">
         <v>19</v>
       </c>
@@ -1696,7 +1641,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="29" t="s">
         <v>21</v>
       </c>
@@ -1708,7 +1653,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="25"/>
       <c r="C14" s="20"/>
       <c r="D14" s="18"/>
@@ -1718,7 +1663,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="2:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="53" t="s">
         <v>24</v>
       </c>
@@ -1734,7 +1679,7 @@
       </c>
       <c r="H15" s="30"/>
     </row>
-    <row r="16" spans="2:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="31" t="s">
         <v>28</v>
       </c>
@@ -1751,7 +1696,7 @@
       </c>
       <c r="H16" s="22"/>
     </row>
-    <row r="17" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B17" s="36" t="s">
         <v>29</v>
       </c>
@@ -1768,7 +1713,7 @@
       </c>
       <c r="H17" s="22"/>
     </row>
-    <row r="18" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B18" s="36" t="s">
         <v>30</v>
       </c>
@@ -1785,7 +1730,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B19" s="36"/>
       <c r="C19" s="37"/>
       <c r="D19" s="38"/>
@@ -1796,7 +1741,7 @@
       </c>
       <c r="H19" s="30"/>
     </row>
-    <row r="20" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B20" s="36"/>
       <c r="C20" s="37"/>
       <c r="D20" s="38"/>
@@ -1807,7 +1752,7 @@
       </c>
       <c r="H20" s="30"/>
     </row>
-    <row r="21" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="36"/>
       <c r="C21" s="37"/>
       <c r="D21" s="38"/>
@@ -1818,7 +1763,7 @@
       </c>
       <c r="H21" s="30"/>
     </row>
-    <row r="22" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="36"/>
       <c r="C22" s="37"/>
       <c r="D22" s="38"/>
@@ -1829,7 +1774,7 @@
       </c>
       <c r="H22" s="30"/>
     </row>
-    <row r="23" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="36"/>
       <c r="C23" s="37"/>
       <c r="D23" s="38"/>
@@ -1840,7 +1785,7 @@
       </c>
       <c r="H23" s="30"/>
     </row>
-    <row r="24" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="36"/>
       <c r="C24" s="37"/>
       <c r="D24" s="38"/>
@@ -1851,7 +1796,7 @@
       </c>
       <c r="H24" s="30"/>
     </row>
-    <row r="25" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="36"/>
       <c r="C25" s="37"/>
       <c r="D25" s="38"/>
@@ -1862,7 +1807,7 @@
       </c>
       <c r="H25" s="30"/>
     </row>
-    <row r="26" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="36"/>
       <c r="C26" s="37"/>
       <c r="D26" s="38"/>
@@ -1873,7 +1818,7 @@
       </c>
       <c r="H26" s="30"/>
     </row>
-    <row r="27" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="36"/>
       <c r="C27" s="37"/>
       <c r="D27" s="38"/>
@@ -1884,7 +1829,7 @@
       </c>
       <c r="H27" s="30"/>
     </row>
-    <row r="28" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="36"/>
       <c r="C28" s="37"/>
       <c r="D28" s="38"/>
@@ -1895,7 +1840,7 @@
       </c>
       <c r="H28" s="30"/>
     </row>
-    <row r="29" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="36"/>
       <c r="C29" s="37"/>
       <c r="D29" s="38"/>
@@ -1906,7 +1851,7 @@
       </c>
       <c r="H29" s="30"/>
     </row>
-    <row r="30" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="41"/>
       <c r="C30" s="42"/>
       <c r="D30" s="38"/>
@@ -1917,7 +1862,7 @@
       </c>
       <c r="H30" s="30"/>
     </row>
-    <row r="31" spans="2:8" s="8" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:8" s="8" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B31" s="63" t="s">
         <v>32</v>
       </c>
@@ -1932,7 +1877,7 @@
       </c>
       <c r="H31" s="22"/>
     </row>
-    <row r="32" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="23"/>
       <c r="C32" s="16"/>
       <c r="D32" s="64" t="s">
@@ -1946,7 +1891,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B33" s="23"/>
       <c r="C33" s="16"/>
       <c r="D33" s="23" t="s">
@@ -1959,7 +1904,7 @@
       </c>
       <c r="H33" s="22"/>
     </row>
-    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:8" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B34" s="47"/>
       <c r="C34" s="48"/>
       <c r="D34" s="49" t="s">
@@ -1974,7 +1919,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B35" s="18"/>
       <c r="C35" s="16"/>
       <c r="D35" s="50"/>
@@ -1984,7 +1929,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="36" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B36" s="16"/>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
@@ -1992,7 +1937,7 @@
       <c r="F36" s="16"/>
       <c r="H36" s="22"/>
     </row>
-    <row r="37" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="65" t="s">
         <v>40</v>
       </c>
@@ -2002,7 +1947,7 @@
       <c r="F37" s="65"/>
       <c r="H37" s="30"/>
     </row>
-    <row r="38" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="61" t="s">
         <v>41</v>
       </c>
@@ -2014,14 +1959,14 @@
         <v>42</v>
       </c>
     </row>
-    <row r="39" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="H39" s="51"/>
     </row>
-    <row r="40" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="42" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="43" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="44" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="E2:F2"/>
@@ -2038,57 +1983,56 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="H3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B13" r:id="rId1" xr:uid="{7D67FB74-A230-4402-B761-380236A85021}"/>
     <hyperlink ref="H4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="B13" r:id="rId3" xr:uid="{7D67FB74-A230-4402-B761-380236A85021}"/>
+    <hyperlink ref="H3" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.5" footer="0.25"/>
   <pageSetup fitToHeight="0" orientation="portrait" r:id="rId4"/>
-  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="78.69921875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="78.6640625" style="1" customWidth="1"/>
     <col min="2" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:2" s="6" customFormat="1" ht="15.6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="1:2" s="6" customFormat="1" ht="16" x14ac:dyDescent="0.15">
       <c r="A2" s="59" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="11"/>
     </row>
-    <row r="3" spans="1:2" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="10"/>
     </row>
-    <row r="4" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:2" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:2" ht="25.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="5" spans="1:2" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="64" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="9"/>
     </row>
-    <row r="8" spans="1:2" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="82.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
         <v>45</v>
       </c>
@@ -2104,24 +2048,13 @@
 </worksheet>
 </file>
 
-<file path=customXml/item12.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2442,28 +2375,35 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item33.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps12.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D626D1C8-EC9A-4213-BF72-F97E82B4EAAA}">
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C42C6076-3E7F-4885-A017-B36671B5853A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{368254F9-4B70-4B70-9250-7541232C303C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2484,10 +2424,14 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps33.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C42C6076-3E7F-4885-A017-B36671B5853A}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D626D1C8-EC9A-4213-BF72-F97E82B4EAAA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>